<commit_message>
Document final bounded UX parity reruns
</commit_message>
<xml_diff>
--- a/tools/foreground-captures/excel-data-validation-dropdown-prepared/prepared-validation-list.xlsx
+++ b/tools/foreground-captures/excel-data-validation-dropdown-prepared/prepared-validation-list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\anton\Documents\Claude\FreeX\.worktrees\ux-parity-s2s7-dialog-dropdown-edge-20260610b\tools\foreground-captures\excel-data-validation-dropdown-prepared\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\anton\Documents\Claude\FreeX\.worktrees\main-integration-20260607b\tools\foreground-captures\excel-data-validation-dropdown-prepared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B27DB2DF-CBC0-4453-85F3-24D8BBCFBE87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5C12590-8411-4503-8A51-46DB9E278553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18000" windowHeight="14400" xr2:uid="{D5B11212-9666-42A9-A118-2261D45A9462}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18000" windowHeight="14400" xr2:uid="{17EB9662-BDD2-46B5-941C-2D0E6F9A917B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -419,7 +419,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C497FDCB-1DC5-4078-BFCE-A257003D9677}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7F8123-36DD-44DB-9AA5-691FBE717A3C}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -452,7 +452,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{66C733B4-4CDF-47F0-9490-8105109F503C}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{62FFA575-8676-400C-B9A7-841707AE8A25}">
       <formula1>"North,South,West"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Harden Excel foreground S2 S7 evidence
</commit_message>
<xml_diff>
--- a/tools/foreground-captures/excel-data-validation-dropdown-prepared/prepared-validation-list.xlsx
+++ b/tools/foreground-captures/excel-data-validation-dropdown-prepared/prepared-validation-list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\anton\Documents\Claude\FreeX\.worktrees\main-integration-20260607b\tools\foreground-captures\excel-data-validation-dropdown-prepared\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\anton\Documents\Claude\FreeX\.worktrees\excel-foreground-s2s7-20260611\tools\foreground-captures\excel-data-validation-dropdown-prepared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5C12590-8411-4503-8A51-46DB9E278553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7E8BC82-1AF9-49CF-AFF1-74AB5A873DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18000" windowHeight="14400" xr2:uid="{17EB9662-BDD2-46B5-941C-2D0E6F9A917B}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18000" windowHeight="14400" xr2:uid="{FB8CE585-CB87-4FD3-831E-0D435FE75E62}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -419,7 +419,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7F8123-36DD-44DB-9AA5-691FBE717A3C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E11AB18D-E525-49EB-99AF-627B3A84840C}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -452,7 +452,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{62FFA575-8676-400C-B9A7-841707AE8A25}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{5B2E70C8-D4AD-4063-8417-3629ADB153BA}">
       <formula1>"North,South,West"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>